<commit_message>
cambios de programa principal y funcion 6
</commit_message>
<xml_diff>
--- a/Datos/Casos resueltos.xlsx
+++ b/Datos/Casos resueltos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -670,6 +670,123 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Florencia Romero</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Femenino</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pelo castaño oscuro rizado, ojos verdes, tez clara</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Cuyo</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Tiene un tatuaje de un león en el hombro</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paula Benítez</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>55</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Femenino</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pelo pelirrojo rizado, ojos celestes, tez morena</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>GBA Sur</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Tiene un tatuaje de un fénix en el brazo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gonzalo Silva</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>32</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Masculino</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Pelo rapado, ojos celestes, tez clara</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>GBA Oeste</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Usa ropa oversize en tonos oscuros</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>